<commit_message>
Acrescentei a opção de despacho
</commit_message>
<xml_diff>
--- a/modelos/OdP's de cada odp.xlsx
+++ b/modelos/OdP's de cada odp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E9A9D16-9D8A-464E-8459-46F2CE1235DE}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E4E1B3C-AD99-4FCA-92BE-55B370D6EBA9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>DATA:</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t xml:space="preserve">DATA DA PESAGEM </t>
+  </si>
+  <si>
+    <t>DESPACHO</t>
   </si>
 </sst>
 </file>
@@ -164,7 +167,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -402,6 +405,32 @@
       <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -409,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -525,6 +554,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -541,10 +579,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -748,31 +782,32 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AG6"/>
+  <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.42578125" customWidth="1"/>
     <col min="2" max="3" width="22.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="23.28515625" customWidth="1"/>
-    <col min="9" max="9" width="23.85546875" customWidth="1"/>
-    <col min="10" max="10" width="29.140625" customWidth="1"/>
-    <col min="11" max="11" width="51.28515625" customWidth="1"/>
-    <col min="12" max="12" width="19.85546875" customWidth="1"/>
-    <col min="13" max="13" width="21.5703125" customWidth="1"/>
-    <col min="14" max="14" width="75.7109375" customWidth="1"/>
-    <col min="15" max="15" width="21" customWidth="1"/>
-    <col min="16" max="17" width="18.7109375" customWidth="1"/>
-    <col min="18" max="19" width="18.85546875" customWidth="1"/>
-    <col min="20" max="20" width="26.42578125" customWidth="1"/>
-    <col min="21" max="21" width="17.140625" customWidth="1"/>
-    <col min="22" max="23" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="17.42578125" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="23.28515625" customWidth="1"/>
+    <col min="10" max="10" width="23.85546875" customWidth="1"/>
+    <col min="11" max="11" width="29.140625" customWidth="1"/>
+    <col min="12" max="12" width="51.28515625" customWidth="1"/>
+    <col min="13" max="13" width="19.85546875" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" customWidth="1"/>
+    <col min="15" max="15" width="75.7109375" customWidth="1"/>
+    <col min="16" max="16" width="21" customWidth="1"/>
+    <col min="17" max="18" width="18.7109375" customWidth="1"/>
+    <col min="19" max="20" width="18.85546875" customWidth="1"/>
+    <col min="21" max="21" width="26.42578125" customWidth="1"/>
+    <col min="22" max="22" width="17.140625" customWidth="1"/>
+    <col min="23" max="24" width="21.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="14"/>
       <c r="B1" s="15"/>
       <c r="C1" s="24" t="s">
@@ -797,9 +832,10 @@
       <c r="T1" s="25"/>
       <c r="U1" s="25"/>
       <c r="V1" s="25"/>
-      <c r="W1" s="26"/>
+      <c r="W1" s="25"/>
+      <c r="X1" s="26"/>
     </row>
-    <row r="2" spans="1:33" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="16"/>
       <c r="B2" s="17"/>
       <c r="C2" s="27"/>
@@ -822,28 +858,29 @@
       <c r="T2" s="28"/>
       <c r="U2" s="28"/>
       <c r="V2" s="28"/>
-      <c r="W2" s="29"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="29"/>
     </row>
-    <row r="3" spans="1:33" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="18"/>
       <c r="B3" s="19"/>
       <c r="C3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="38"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="37"/>
       <c r="I3" s="38"/>
       <c r="J3" s="38"/>
       <c r="K3" s="38"/>
       <c r="L3" s="38"/>
-      <c r="M3" s="39"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="31"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="30"/>
       <c r="P3" s="31"/>
       <c r="Q3" s="31"/>
       <c r="R3" s="31"/>
@@ -851,9 +888,10 @@
       <c r="T3" s="31"/>
       <c r="U3" s="31"/>
       <c r="V3" s="31"/>
-      <c r="W3" s="32"/>
+      <c r="W3" s="31"/>
+      <c r="X3" s="32"/>
     </row>
-    <row r="4" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="20"/>
       <c r="B4" s="21"/>
       <c r="C4" s="36"/>
@@ -863,12 +901,12 @@
       <c r="G4" s="36"/>
       <c r="H4" s="36"/>
       <c r="I4" s="36"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="13"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="12"/>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="34"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="33"/>
       <c r="P4" s="34"/>
       <c r="Q4" s="34"/>
       <c r="R4" s="34"/>
@@ -876,9 +914,10 @@
       <c r="T4" s="34"/>
       <c r="U4" s="34"/>
       <c r="V4" s="34"/>
-      <c r="W4" s="35"/>
+      <c r="W4" s="34"/>
+      <c r="X4" s="35"/>
     </row>
-    <row r="5" spans="1:33" ht="37.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:34" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A5" s="22"/>
       <c r="B5" s="23"/>
       <c r="C5" s="7" t="s">
@@ -887,89 +926,93 @@
       <c r="D5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="42" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="J5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="K5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="L5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="M5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="N5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="O5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="P5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="P5" s="6" t="s">
+      <c r="Q5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="R5" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="R5" s="5" t="s">
+      <c r="S5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="S5" s="5" t="s">
+      <c r="T5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T5" s="5" t="s">
+      <c r="U5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="U5" s="5" t="s">
+      <c r="V5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="V5" s="5" t="s">
+      <c r="W5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="W5" s="6" t="s">
+      <c r="X5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
       <c r="AB5" s="1"/>
-      <c r="AC5" s="2"/>
+      <c r="AC5" s="1"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
       <c r="AF5" s="2"/>
       <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
     </row>
-    <row r="6" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="N6" s="3"/>
+    <row r="6" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="J4:M4"/>
+  <mergeCells count="8">
+    <mergeCell ref="K4:N4"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:B5"/>
-    <mergeCell ref="C1:W2"/>
-    <mergeCell ref="N3:W4"/>
-    <mergeCell ref="C4:I4"/>
-    <mergeCell ref="G3:M3"/>
+    <mergeCell ref="C1:X2"/>
+    <mergeCell ref="O3:X4"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="H3:N3"/>
+    <mergeCell ref="D3:E3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Acrescentei a opção de acrescentar novas OdP's ao longo do dia
</commit_message>
<xml_diff>
--- a/modelos/OdP's de cada odp.xlsx
+++ b/modelos/OdP's de cada odp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E4E1B3C-AD99-4FCA-92BE-55B370D6EBA9}"/>
+  <xr:revisionPtr revIDLastSave="227" documentId="11_69D1BB207A00D00DEC82CC547798B416B8469308" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{485BC9A5-7DC0-4BC0-996F-FDFEEA29E297}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -465,12 +465,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -561,8 +561,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -579,6 +579,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -872,7 +876,7 @@
       <c r="F3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="10"/>
+      <c r="G3" s="42"/>
       <c r="H3" s="37"/>
       <c r="I3" s="38"/>
       <c r="J3" s="38"/>
@@ -926,10 +930,10 @@
       <c r="D5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="42" t="s">
+      <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="42" t="s">
+      <c r="F5" s="11" t="s">
         <v>3</v>
       </c>
       <c r="G5" s="7" t="s">
@@ -965,7 +969,7 @@
       <c r="Q5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="R5" s="11" t="s">
+      <c r="R5" s="10" t="s">
         <v>22</v>
       </c>
       <c r="S5" s="5" t="s">

</xml_diff>